<commit_message>
Fase di Validazioine nela parte di ricerca dei parametri XGBoost e matrice di confusione
Sistemato la parte dove fermo il processo se l'errore inizia a salire già nella parte in cui riceco i parametri migliori e stampa delle 2 matrici di confiusione
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4_Risultati_GridSearch_XGBoost.xlsx
+++ b/export_dati/04_Step4_Risultati_GridSearch_XGBoost.xlsx
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Accuratezza Media (CV)</t>
+          <t>Accuratezza Media</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -456,16 +456,16 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>95.45%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.0007</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -474,22 +474,22 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="B3" t="n">
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>95.43%</t>
+          <t>95.25%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.0022</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -498,7 +498,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
@@ -508,12 +508,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>95.35%</t>
+          <t>95.05%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -525,19 +525,19 @@
         <v>0.01</v>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>95.33%</t>
+          <t>94.90%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -549,19 +549,19 @@
         <v>0.01</v>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
         <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>95.28%</t>
+          <t>94.80%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.0024</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -570,50 +570,50 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B7" t="n">
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>95.28%</t>
+          <t>94.80%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.0041</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B8" t="n">
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>95.25%</t>
+          <t>94.80%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.0039</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -628,36 +628,36 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>95.22%</t>
+          <t>94.80%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
         <v>300</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>95.20%</t>
+          <t>94.75%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -666,26 +666,26 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B11" t="n">
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>95.10%</t>
+          <t>94.75%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -696,16 +696,16 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>95.10%</t>
+          <t>94.65%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -714,22 +714,22 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C13" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>95.08%</t>
+          <t>94.55%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.0021</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -738,26 +738,26 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="B14" t="n">
         <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>95.08%</t>
+          <t>94.45%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -772,16 +772,16 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>95.07%</t>
+          <t>94.45%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -796,36 +796,36 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>94.95%</t>
+          <t>94.45%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>94.93%</t>
+          <t>94.40%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -834,46 +834,46 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B18" t="n">
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>94.92%</t>
+          <t>94.40%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B19" t="n">
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>94.90%</t>
+          <t>94.35%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -885,91 +885,91 @@
         <v>0.1</v>
       </c>
       <c r="B20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
         <v>200</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>94.88%</t>
+          <t>94.35%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.0026</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>94.85%</t>
+          <t>94.35%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0.0032</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B22" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
         <v>300</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>94.82%</t>
+          <t>94.35%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.0013</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C23" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>94.78%</t>
+          <t>94.25%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.0009</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -978,22 +978,22 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>94.73%</t>
+          <t>94.20%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0.0030</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1002,37 +1002,37 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="B25" t="n">
         <v>6</v>
       </c>
       <c r="C25" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>94.73%</t>
+          <t>94.20%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.0012</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C26" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1041,35 +1041,35 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.0043</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="B27" t="n">
         <v>9</v>
       </c>
       <c r="C27" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>94.18%</t>
+          <t>94.20%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0.0026</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>87.03%</t>
+          <t>88.15%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0.0090</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="F28" t="n">

</xml_diff>

<commit_message>
Codice funzionante con ottimizzazione su dataset di test
usato dataset di test per fare le statistiche, per me sbagliato
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4_Risultati_GridSearch_XGBoost.xlsx
+++ b/export_dati/04_Step4_Risultati_GridSearch_XGBoost.xlsx
@@ -450,17 +450,17 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>98.68%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -477,14 +477,14 @@
         <v>0.05</v>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -501,14 +501,14 @@
         <v>0.05</v>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>95.45%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -517,22 +517,22 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B5" t="n">
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>95.45%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -541,22 +541,22 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>95.45%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -580,7 +580,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>95.45%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -597,14 +597,14 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
         <v>100</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>95.40%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -621,14 +621,14 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
         <v>200</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>95.40%</t>
+          <t>98.66%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -637,12 +637,12 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="B10" t="n">
         <v>6</v>
@@ -652,7 +652,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>95.40%</t>
+          <t>98.65%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -661,22 +661,22 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>95.35%</t>
+          <t>98.64%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -690,17 +690,17 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
         <v>300</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>95.35%</t>
+          <t>98.64%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -714,7 +714,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="B13" t="n">
         <v>9</v>
@@ -724,7 +724,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.64%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -741,14 +741,14 @@
         <v>0.05</v>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
         <v>100</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.64%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -757,22 +757,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.63%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -781,22 +781,22 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="B16" t="n">
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.63%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -805,22 +805,22 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="B17" t="n">
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.63%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -829,22 +829,22 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="B18" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -853,22 +853,22 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="B19" t="n">
         <v>9</v>
       </c>
       <c r="C19" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>95.20%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20">
@@ -885,14 +885,14 @@
         <v>0.05</v>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>95.20%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -901,22 +901,22 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>95.15%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -925,22 +925,22 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="B22" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>95.15%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -949,22 +949,22 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="B23" t="n">
         <v>9</v>
       </c>
       <c r="C23" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>95.15%</t>
+          <t>98.62%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24">
@@ -981,14 +981,14 @@
         <v>0.01</v>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
         <v>200</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>95.10%</t>
+          <t>98.61%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1002,17 +1002,17 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="B25" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>94.80%</t>
+          <t>98.61%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
@@ -1029,14 +1029,14 @@
         <v>0.01</v>
       </c>
       <c r="B26" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C26" t="n">
         <v>100</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>94.10%</t>
+          <t>98.35%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1053,14 +1053,14 @@
         <v>0.01</v>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C27" t="n">
         <v>100</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>93.90%</t>
+          <t>98.32%</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>88.60%</t>
+          <t>97.91%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">

</xml_diff>